<commit_message>
Every grant except QBE buys 133 beds; REAL is Oonchiumpa's offer
Ben, 15 September 2026, afternoon. Brian M. Davis becomes one line of 133 beds at
$750 ($99,750), the 80 beds plus $40,000 facilitation split withdrawn. Tim Fairfax
buys 133 beds each year; the operating-support form is answered as the $288 those
beds hand back. Nobody is asked for the running cost. SEDI leaves the bed stack
because both streams buy capability services only.

The Commonwealth money is corrected from the DEWR outcome letter: one REAL
Innovation Fund offer of $1,695,000 to Oonchiumpa over four years, not executed,
plus a NIAA door with no invitation. Nothing is approved to the applicant and
nothing is counted; the two Commonwealth scenarios that assumed $150,000 approved
and a second tranche are removed.

Asked is now $599,750 across four lines, the gap $136,437, sent asks cover 266 of
400 beds. The ladder loses its facilitation rung and gains the $99,750 lot. The
workbook is regenerated.
</commit_message>
<xml_diff>
--- a/deliverables/finance/funder-model/goods-funder-model-2026-09-15.xlsx
+++ b/deliverables/finance/funder-model/goods-funder-model-2026-09-15.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="871" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="530">
   <si>
     <t>Goods on Country, financial model for funders</t>
   </si>
@@ -836,13 +836,13 @@
     <t>Beds: making 400 of first stock</t>
   </si>
   <si>
-    <t>Brian M. Davis (invited), Snow (not sent). Bed money is asked at the price, so this line over-covers the making cost and the surplus carries the organisation.</t>
+    <t>Tim Fairfax (invited, year one of three), Brian M. Davis (invited), Snow (not sent), each 133 beds at $750. Bed money is asked at the price, so this line over-covers the making cost and the surplus carries the organisation.</t>
   </si>
   <si>
     <t>Organisation: running it, and the freight and facilitation it absorbs</t>
   </si>
   <si>
-    <t>Tim Fairfax (invited, year one of three) and the facilitation half of the Brian M. Davis invitation. The rest is carried by 400 beds at the contribution.</t>
+    <t>Nobody is asked for this line (Ben, 15 September 2026). It is carried by 400 beds at the contribution, and by trade beyond them.</t>
   </si>
   <si>
     <t>The year needs</t>
@@ -893,25 +893,16 @@
     <t>Tim Fairfax Family Foundation</t>
   </si>
   <si>
-    <t>operating</t>
-  </si>
-  <si>
     <t>invited</t>
   </si>
   <si>
-    <t>Katie Norman, 31 August 2026: a three-year grant of $300,000 in three equal payments, naming the resilience of organisations. Year one is $100,000 and it belongs on the operating line alone.</t>
+    <t>Katie Norman, 31 August 2026: a three-year grant of $300,000 in three equal payments under General Operating Support. Ben, 15 September 2026: year one buys 133 beds at $750; the organisation's share is the contribution those beds hand back. The form's operating framing is a flag, not a job.</t>
   </si>
   <si>
     <t>Brian M. Davis Charitable Foundation</t>
   </si>
   <si>
-    <t>Miranda Campbell, 1 September 2026: up to $100,000 for twelve months. 80 beds at $750.</t>
-  </si>
-  <si>
-    <t>facilitation</t>
-  </si>
-  <si>
-    <t>The other half of the same invitation. Facilitation in four communities.</t>
+    <t>Miranda Campbell, 1 September 2026: up to $100,000 for twelve months. Ben, 15 September 2026: 133 beds at $750, facilitation inside, one budget line. The old 80 beds plus $40,000 facilitation split is withdrawn.</t>
   </si>
   <si>
     <t>Snow Foundation</t>
@@ -920,7 +911,7 @@
     <t>not-sent</t>
   </si>
   <si>
-    <t>Ben wrote $100,000 on 10 September and ruled it counts as beds. The ask has not been sent.</t>
+    <t>Ben wrote $100,000 on 10 September and ruled it counts as beds, 133 at $750. The ask has not been sent.</t>
   </si>
   <si>
     <t>Dusseldorp Forum</t>
@@ -953,7 +944,7 @@
     <t>No Snow, no Dusseldorp</t>
   </si>
   <si>
-    <t>Five lines, all grants. Dusseldorp and SEFA are outside the ask.</t>
+    <t>Four lines, all grants. Dusseldorp and SEFA are outside the ask.</t>
   </si>
   <si>
     <t>Secured</t>
@@ -1013,7 +1004,7 @@
     <t>Beds at the contribution, after making, freight and facilitation.</t>
   </si>
   <si>
-    <t>Against running alone, because the contribution already carries the freight and facilitation. Tim Fairfax year one goes against this.</t>
+    <t>Against running alone, because the contribution already carries the freight and facilitation. No grant goes against this line; it is the running short that trade or debt has to cover.</t>
   </si>
   <si>
     <t>Monthly cash, July 2026 to June 2027. A scenario laid out from the Inputs sheet. Nobody has forecast these months. Built 2026-09-15.</t>
@@ -1067,16 +1058,10 @@
     <t>Scenario month only. No receipt date exists. Applying; closes 25 September.</t>
   </si>
   <si>
-    <t>Grants for beds (Brian M. Davis)</t>
-  </si>
-  <si>
-    <t>Scenario month only. No receipt date exists. Invited; board 19 November.</t>
-  </si>
-  <si>
-    <t>Grants for facilitation (Brian M. Davis)</t>
-  </si>
-  <si>
-    <t>Scenario month only. No receipt date exists. The other half of the same invitation.</t>
+    <t>Grants for beds (Brian M. Davis, 133 beds)</t>
+  </si>
+  <si>
+    <t>Scenario month only. No receipt date exists. Invited; board 19 November. One line, facilitation inside the bed.</t>
   </si>
   <si>
     <t>Grants for beds (Snow, Dusseldorp)</t>
@@ -1085,10 +1070,10 @@
     <t>Untimed and zero. Neither ask has been sent, so no month is honest.</t>
   </si>
   <si>
-    <t>Grants for operations (Tim Fairfax, year one)</t>
-  </si>
-  <si>
-    <t>Scenario month only. No receipt date exists. Invited; SmartyGrants closes 9 October, board late November.</t>
+    <t>Grants for beds (Tim Fairfax, year one, 133 beds)</t>
+  </si>
+  <si>
+    <t>Scenario month only. No receipt date exists. Invited; SmartyGrants closes 9 October, board late November. Ben, 15 September 2026: buys beds, not the running cost.</t>
   </si>
   <si>
     <t>Loan drawn (SEFA)</t>
@@ -1407,9 +1392,6 @@
   </si>
   <si>
     <t>ASKS[3].amountAud</t>
-  </si>
-  <si>
-    <t>ASKS[4].amountAud</t>
   </si>
   <si>
     <t>BEDS_AT_COST_AUD</t>
@@ -3737,7 +3719,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -3814,8 +3796,8 @@
         <v>104962.66666666667</v>
       </c>
       <c r="C5" s="8">
-        <f>SUM(B13,B15)</f>
-        <v>160000</v>
+        <f>SUM(B12,B13,B14)</f>
+        <v>299750</v>
       </c>
       <c r="D5" s="8">
         <f>MAX(0,B5-C5)</f>
@@ -3834,12 +3816,11 @@
         <v>331224</v>
       </c>
       <c r="C6" s="8">
-        <f>SUM(B12,B14)</f>
-        <v>140000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="8">
         <f>MAX(0,B6-C6)</f>
-        <v>191224</v>
+        <v>331224</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>274</v>
@@ -3855,11 +3836,11 @@
       </c>
       <c r="C7" s="12">
         <f>SUM(C4,C5,C6)</f>
-        <v>600000</v>
+        <v>599750</v>
       </c>
       <c r="D7" s="12">
         <f>B7-C7</f>
-        <v>136186.66666666674</v>
+        <v>136436.66666666674</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>276</v>
@@ -3930,60 +3911,62 @@
         <v>100000</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>287</v>
+      <c r="E12" s="6">
+        <f>FLOOR(B12/'Inputs'!C4,1)</f>
+        <v>133</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>288</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B13" s="5">
-        <v>60000</v>
+        <v>99750</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E13" s="6">
         <f>FLOOR(B13/'Inputs'!C4,1)</f>
-        <v>80</v>
+        <v>133</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>288</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B14" s="5">
-        <v>40000</v>
+        <v>100000</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>287</v>
+      <c r="E14" s="6">
+        <f>FLOOR(B14/'Inputs'!C4,1)</f>
+        <v>133</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>288</v>
@@ -3997,20 +3980,20 @@
         <v>298</v>
       </c>
       <c r="B15" s="5">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="E15" s="6">
         <f>FLOOR(B15/'Inputs'!C4,1)</f>
-        <v>133</v>
+        <v>66</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>288</v>
+        <v>299</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>300</v>
@@ -4020,267 +4003,243 @@
       <c r="A16" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="B16" s="5">
-        <v>50000</v>
+      <c r="B16" s="13">
+        <v>200000</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="E16" s="6">
-        <f>FLOOR(B16/'Inputs'!C4,1)</f>
-        <v>66</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>302</v>
-      </c>
       <c r="G16" s="2" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="B17" s="13">
-        <v>200000</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D17" s="2" t="s">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>305</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="G17" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
-        <v>308</v>
-      </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
+      <c r="D19" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="B20" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B20" s="12">
+        <f>SUM(B11,B12,B13,B14)</f>
+        <v>599750</v>
+      </c>
+      <c r="C20" s="12">
+        <f>SUM(B11,B12,B13)</f>
+        <v>499750</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="B21" s="5">
+        <v>0</v>
+      </c>
+      <c r="C21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="B21" s="12">
-        <f>SUM(B11,B12,B13,B14,B15)</f>
-        <v>600000</v>
-      </c>
-      <c r="C21" s="12">
-        <f>SUM(B11,B12,B13,B14)</f>
-        <v>500000</v>
-      </c>
-      <c r="G21" s="3" t="s">
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+      <c r="B22" s="12">
+        <f>B7-B20</f>
+        <v>136436.66666666674</v>
+      </c>
+      <c r="C22" s="12">
+        <f>B7-C20</f>
+        <v>236436.66666666674</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>312</v>
-      </c>
-      <c r="B22" s="5">
-        <v>0</v>
-      </c>
-      <c r="C22" s="5">
-        <v>0</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="B23" s="11">
+        <f>FLOOR(SUM(B12,B13,B14)/'Inputs'!C4,1)</f>
+        <v>399</v>
+      </c>
+      <c r="C23" s="11">
+        <f>FLOOR(SUM(B12,B13)/'Inputs'!C4,1)</f>
+        <v>266</v>
+      </c>
+      <c r="G23" s="3" t="s">
         <v>314</v>
-      </c>
-      <c r="B23" s="12">
-        <f>B7-B21</f>
-        <v>136186.66666666674</v>
-      </c>
-      <c r="C23" s="12">
-        <f>B7-C21</f>
-        <v>236186.66666666674</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="B24" s="11">
+        <f>'Inputs'!C20-C23</f>
+        <v>134</v>
+      </c>
+      <c r="C24" s="11">
+        <f>'Inputs'!C20-C23</f>
+        <v>134</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>316</v>
-      </c>
-      <c r="B24" s="11">
-        <f>FLOOR(SUM(B13,B15)/'Inputs'!C4,1)</f>
-        <v>213</v>
-      </c>
-      <c r="C24" s="11">
-        <f>FLOOR(SUM(B13)/'Inputs'!C4,1)</f>
-        <v>80</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="B25" s="11">
+        <f>'Inputs'!C20-B23</f>
+        <v>1</v>
+      </c>
+      <c r="C25" s="11">
+        <f>'Inputs'!C20-C23</f>
+        <v>134</v>
+      </c>
+      <c r="G25" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="B25" s="11">
-        <f>'Inputs'!C20-C24</f>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="B26" s="8">
+        <v>331224</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>320</v>
-      </c>
-      <c r="C25" s="11">
-        <f>'Inputs'!C20-C24</f>
-        <v>320</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>320</v>
-      </c>
-      <c r="B26" s="11">
-        <f>'Inputs'!C20-B24</f>
-        <v>187</v>
-      </c>
-      <c r="C26" s="11">
-        <f>'Inputs'!C20-C24</f>
-        <v>320</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="B27" s="8">
+        <v>194787.3333333333</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="B27" s="8">
-        <v>191224</v>
-      </c>
-      <c r="G27" s="2" t="s">
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="2" t="s">
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="B28" s="8">
-        <v>55037.33333333333</v>
-      </c>
-      <c r="G28" s="2" t="s">
+      <c r="B31" s="8">
+        <f>'Inputs'!C37</f>
+        <v>331224</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>325</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>326</v>
-      </c>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B32" s="8">
-        <f>'Inputs'!C37</f>
-        <v>331224</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="B33" s="8">
         <f>'Inputs'!C38</f>
         <v>115037.33333333333</v>
       </c>
-      <c r="G33" s="2" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
+      <c r="G32" s="2" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B34" s="12">
+      <c r="B33" s="12">
         <f>'Inputs'!C39</f>
         <v>136186.6666666667</v>
       </c>
-      <c r="G34" s="3" t="s">
-        <v>331</v>
+      <c r="G33" s="3" t="s">
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -4291,7 +4250,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -4302,7 +4261,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -4310,43 +4269,43 @@
         <v>240</v>
       </c>
       <c r="B2" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>342</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>343</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>344</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>345</v>
       </c>
       <c r="O2" s="3" t="s">
         <v>16</v>
@@ -4354,7 +4313,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -4373,7 +4332,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="B4" s="5">
         <v>0</v>
@@ -4416,12 +4375,12 @@
         <v>300000</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>
@@ -4439,7 +4398,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="5">
-        <v>60000</v>
+        <v>99750</v>
       </c>
       <c r="H5" s="5">
         <v>0</v>
@@ -4461,15 +4420,15 @@
       </c>
       <c r="N5" s="5">
         <f>SUM(B5:M5)</f>
-        <v>60000</v>
+        <v>99750</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B6" s="5">
         <v>0</v>
@@ -4487,7 +4446,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="5">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="H6" s="5">
         <v>0</v>
@@ -4509,15 +4468,15 @@
       </c>
       <c r="N6" s="5">
         <f>SUM(B6:M6)</f>
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B7" s="5">
         <v>0</v>
@@ -4535,7 +4494,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="5">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="H7" s="5">
         <v>0</v>
@@ -4557,15 +4516,15 @@
       </c>
       <c r="N7" s="5">
         <f>SUM(B7:M7)</f>
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="O7" s="2" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B8" s="5">
         <v>0</v>
@@ -4583,7 +4542,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="5">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5">
         <v>0</v>
@@ -4605,21 +4564,23 @@
       </c>
       <c r="N8" s="5">
         <f>SUM(B8:M8)</f>
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="O8" s="2" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B9" s="5">
-        <v>0</v>
+        <f>SUM('Inputs'!C57)</f>
+        <v>30000</v>
       </c>
       <c r="C9" s="5">
-        <v>0</v>
+        <f>SUM('Inputs'!C58)</f>
+        <v>80000</v>
       </c>
       <c r="D9" s="5">
         <v>0</v>
@@ -4653,144 +4614,143 @@
       </c>
       <c r="N9" s="5">
         <f>SUM(B9:M9)</f>
-        <v>0</v>
+        <v>110000</v>
       </c>
       <c r="O9" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>356</v>
+      </c>
+      <c r="B10" s="12">
+        <f>SUM(B4:B9)</f>
+        <v>30000</v>
+      </c>
+      <c r="C10" s="12">
+        <f>SUM(C4:C9)</f>
+        <v>80000</v>
+      </c>
+      <c r="D10" s="12">
+        <f>SUM(D4:D9)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="12">
+        <f>SUM(E4:E9)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="12">
+        <f>SUM(F4:F9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="12">
+        <f>SUM(G4:G9)</f>
+        <v>499750</v>
+      </c>
+      <c r="H10" s="12">
+        <f>SUM(H4:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="12">
+        <f>SUM(I4:I9)</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="12">
+        <f>SUM(J4:J9)</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="12">
+        <f>SUM(K4:K9)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="12">
+        <f>SUM(L4:L9)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="12">
+        <f>SUM(M4:M9)</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="12">
+        <f>SUM(B10:M10)</f>
+        <v>609750</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="B10" s="5">
-        <f>SUM('Inputs'!C57)</f>
-        <v>30000</v>
-      </c>
-      <c r="C10" s="5">
-        <f>SUM('Inputs'!C58)</f>
-        <v>80000</v>
-      </c>
-      <c r="D10" s="5">
-        <v>0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="5">
-        <v>0</v>
-      </c>
-      <c r="I10" s="5">
-        <v>0</v>
-      </c>
-      <c r="J10" s="5">
-        <v>0</v>
-      </c>
-      <c r="K10" s="5">
-        <v>0</v>
-      </c>
-      <c r="L10" s="5">
-        <v>0</v>
-      </c>
-      <c r="M10" s="5">
-        <v>0</v>
-      </c>
-      <c r="N10" s="5">
-        <f>SUM(B10:M10)</f>
-        <v>110000</v>
-      </c>
-      <c r="O10" s="2" t="s">
+      <c r="B12" s="8">
+        <v>0</v>
+      </c>
+      <c r="C12" s="8">
+        <v>0</v>
+      </c>
+      <c r="D12" s="8">
+        <v>0</v>
+      </c>
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
+      <c r="F12" s="8">
+        <v>0</v>
+      </c>
+      <c r="G12" s="8">
+        <f>'Inputs'!C45</f>
+        <v>300000</v>
+      </c>
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8">
+        <v>0</v>
+      </c>
+      <c r="J12" s="8">
+        <v>0</v>
+      </c>
+      <c r="K12" s="8">
+        <v>0</v>
+      </c>
+      <c r="L12" s="8">
+        <v>0</v>
+      </c>
+      <c r="M12" s="8">
+        <v>0</v>
+      </c>
+      <c r="N12" s="8">
+        <f>SUM(B12:M12)</f>
+        <v>300000</v>
+      </c>
+      <c r="O12" s="2" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="B11" s="12">
-        <f>SUM(B4:B10)</f>
-        <v>30000</v>
-      </c>
-      <c r="C11" s="12">
-        <f>SUM(C4:C10)</f>
-        <v>80000</v>
-      </c>
-      <c r="D11" s="12">
-        <f>SUM(D4:D10)</f>
-        <v>0</v>
-      </c>
-      <c r="E11" s="12">
-        <f>SUM(E4:E10)</f>
-        <v>0</v>
-      </c>
-      <c r="F11" s="12">
-        <f>SUM(F4:F10)</f>
-        <v>0</v>
-      </c>
-      <c r="G11" s="12">
-        <f>SUM(G4:G10)</f>
-        <v>500000</v>
-      </c>
-      <c r="H11" s="12">
-        <f>SUM(H4:H10)</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="12">
-        <f>SUM(I4:I10)</f>
-        <v>0</v>
-      </c>
-      <c r="J11" s="12">
-        <f>SUM(J4:J10)</f>
-        <v>0</v>
-      </c>
-      <c r="K11" s="12">
-        <f>SUM(K4:K10)</f>
-        <v>0</v>
-      </c>
-      <c r="L11" s="12">
-        <f>SUM(L4:L10)</f>
-        <v>0</v>
-      </c>
-      <c r="M11" s="12">
-        <f>SUM(M4:M10)</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="12">
-        <f>SUM(B11:M11)</f>
-        <v>610000</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4"/>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="B13" s="8">
         <v>0</v>
@@ -4808,503 +4768,454 @@
         <v>0</v>
       </c>
       <c r="G13" s="8">
-        <f>'Inputs'!C45</f>
-        <v>300000</v>
+        <v>0</v>
       </c>
       <c r="H13" s="8">
-        <v>0</v>
+        <f>'Inputs'!C50*'Inputs'!C15</f>
+        <v>25191.04</v>
       </c>
       <c r="I13" s="8">
-        <v>0</v>
+        <f>'Inputs'!C50*'Inputs'!C15</f>
+        <v>25191.04</v>
       </c>
       <c r="J13" s="8">
-        <v>0</v>
+        <f>'Inputs'!C50*'Inputs'!C15</f>
+        <v>25191.04</v>
       </c>
       <c r="K13" s="8">
-        <v>0</v>
+        <f>'Inputs'!C50*'Inputs'!C15</f>
+        <v>25191.04</v>
       </c>
       <c r="L13" s="8">
-        <v>0</v>
+        <f>('Inputs'!C20-4*'Inputs'!C50)*'Inputs'!C15</f>
+        <v>4198.506666666667</v>
       </c>
       <c r="M13" s="8">
         <v>0</v>
       </c>
       <c r="N13" s="8">
         <f>SUM(B13:M13)</f>
-        <v>300000</v>
+        <v>104962.66666666667</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="C14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="D14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="E14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="F14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="G14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="H14" s="8">
-        <f>'Inputs'!C50*'Inputs'!C15</f>
-        <v>25191.04</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="I14" s="8">
-        <f>'Inputs'!C50*'Inputs'!C15</f>
-        <v>25191.04</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="J14" s="8">
-        <f>'Inputs'!C50*'Inputs'!C15</f>
-        <v>25191.04</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="K14" s="8">
-        <f>'Inputs'!C50*'Inputs'!C15</f>
-        <v>25191.04</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="L14" s="8">
-        <f>('Inputs'!C20-4*'Inputs'!C50)*'Inputs'!C15</f>
-        <v>4198.506666666667</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="M14" s="8">
-        <v>0</v>
+        <f>'Inputs'!C28/'Inputs'!C24</f>
+        <v>3333.3333333333335</v>
       </c>
       <c r="N14" s="8">
         <f>SUM(B14:M14)</f>
-        <v>104962.66666666667</v>
+        <v>40000</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>368</v>
+        <v>123</v>
       </c>
       <c r="B15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="C15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="D15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="E15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="F15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="G15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="H15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="I15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="J15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="K15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="L15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="M15" s="8">
-        <f>'Inputs'!C28/'Inputs'!C24</f>
-        <v>3333.3333333333335</v>
+        <f>'Inputs'!C36/'Inputs'!C24</f>
+        <v>20935.333333333332</v>
       </c>
       <c r="N15" s="8">
         <f>SUM(B15:M15)</f>
-        <v>40000</v>
+        <v>251224</v>
       </c>
       <c r="O15" s="2" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>123</v>
+        <v>366</v>
       </c>
       <c r="B16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="C16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="D16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="E16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="F16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="G16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="H16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <f>'Inputs'!C50*'Inputs'!C16</f>
+        <v>9600</v>
       </c>
       <c r="I16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <f>'Inputs'!C50*'Inputs'!C16</f>
+        <v>9600</v>
       </c>
       <c r="J16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <f>'Inputs'!C50*'Inputs'!C16</f>
+        <v>9600</v>
       </c>
       <c r="K16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <f>'Inputs'!C50*'Inputs'!C16</f>
+        <v>9600</v>
       </c>
       <c r="L16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <f>('Inputs'!C20-4*'Inputs'!C50)*'Inputs'!C16</f>
+        <v>1600</v>
       </c>
       <c r="M16" s="8">
-        <f>'Inputs'!C36/'Inputs'!C24</f>
-        <v>20935.333333333332</v>
+        <v>0</v>
       </c>
       <c r="N16" s="8">
         <f>SUM(B16:M16)</f>
-        <v>251224</v>
+        <v>40000</v>
       </c>
       <c r="O16" s="2" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="B17" s="12">
+        <f>SUM(B12:B16)</f>
+        <v>24268.666666666664</v>
+      </c>
+      <c r="C17" s="12">
+        <f>SUM(C12:C16)</f>
+        <v>24268.666666666664</v>
+      </c>
+      <c r="D17" s="12">
+        <f>SUM(D12:D16)</f>
+        <v>24268.666666666664</v>
+      </c>
+      <c r="E17" s="12">
+        <f>SUM(E12:E16)</f>
+        <v>24268.666666666664</v>
+      </c>
+      <c r="F17" s="12">
+        <f>SUM(F12:F16)</f>
+        <v>24268.666666666664</v>
+      </c>
+      <c r="G17" s="12">
+        <f>SUM(G12:G16)</f>
+        <v>324268.6666666666</v>
+      </c>
+      <c r="H17" s="12">
+        <f>SUM(H12:H16)</f>
+        <v>59059.706666666665</v>
+      </c>
+      <c r="I17" s="12">
+        <f>SUM(I12:I16)</f>
+        <v>59059.706666666665</v>
+      </c>
+      <c r="J17" s="12">
+        <f>SUM(J12:J16)</f>
+        <v>59059.706666666665</v>
+      </c>
+      <c r="K17" s="12">
+        <f>SUM(K12:K16)</f>
+        <v>59059.706666666665</v>
+      </c>
+      <c r="L17" s="12">
+        <f>SUM(L12:L16)</f>
+        <v>30067.173333333332</v>
+      </c>
+      <c r="M17" s="12">
+        <f>SUM(M12:M16)</f>
+        <v>24268.666666666664</v>
+      </c>
+      <c r="N17" s="12">
+        <f>SUM(B17:M17)</f>
+        <v>736186.6666666667</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="2" t="s">
+      <c r="B19" s="12">
+        <f>B10-B17</f>
+        <v>5731.333333333336</v>
+      </c>
+      <c r="C19" s="12">
+        <f>C10-C17</f>
+        <v>55731.333333333336</v>
+      </c>
+      <c r="D19" s="12">
+        <f>D10-D17</f>
+        <v>-24268.666666666664</v>
+      </c>
+      <c r="E19" s="12">
+        <f>E10-E17</f>
+        <v>-24268.666666666664</v>
+      </c>
+      <c r="F19" s="12">
+        <f>F10-F17</f>
+        <v>-24268.666666666664</v>
+      </c>
+      <c r="G19" s="12">
+        <f>G10-G17</f>
+        <v>175481.33333333337</v>
+      </c>
+      <c r="H19" s="12">
+        <f>H10-H17</f>
+        <v>-59059.706666666665</v>
+      </c>
+      <c r="I19" s="12">
+        <f>I10-I17</f>
+        <v>-59059.706666666665</v>
+      </c>
+      <c r="J19" s="12">
+        <f>J10-J17</f>
+        <v>-59059.706666666665</v>
+      </c>
+      <c r="K19" s="12">
+        <f>K10-K17</f>
+        <v>-59059.706666666665</v>
+      </c>
+      <c r="L19" s="12">
+        <f>L10-L17</f>
+        <v>-30067.173333333332</v>
+      </c>
+      <c r="M19" s="12">
+        <f>M10-M17</f>
+        <v>-24268.666666666664</v>
+      </c>
+      <c r="N19" s="12">
+        <f>SUM(B19:M19)</f>
+        <v>-126436.6666666666</v>
+      </c>
+      <c r="O19" s="3" t="s">
         <v>371</v>
       </c>
-      <c r="B17" s="8">
-        <v>0</v>
-      </c>
-      <c r="C17" s="8">
-        <v>0</v>
-      </c>
-      <c r="D17" s="8">
-        <v>0</v>
-      </c>
-      <c r="E17" s="8">
-        <v>0</v>
-      </c>
-      <c r="F17" s="8">
-        <v>0</v>
-      </c>
-      <c r="G17" s="8">
-        <v>0</v>
-      </c>
-      <c r="H17" s="8">
-        <f>'Inputs'!C50*'Inputs'!C16</f>
-        <v>9600</v>
-      </c>
-      <c r="I17" s="8">
-        <f>'Inputs'!C50*'Inputs'!C16</f>
-        <v>9600</v>
-      </c>
-      <c r="J17" s="8">
-        <f>'Inputs'!C50*'Inputs'!C16</f>
-        <v>9600</v>
-      </c>
-      <c r="K17" s="8">
-        <f>'Inputs'!C50*'Inputs'!C16</f>
-        <v>9600</v>
-      </c>
-      <c r="L17" s="8">
-        <f>('Inputs'!C20-4*'Inputs'!C50)*'Inputs'!C16</f>
-        <v>1600</v>
-      </c>
-      <c r="M17" s="8">
-        <v>0</v>
-      </c>
-      <c r="N17" s="8">
-        <f>SUM(B17:M17)</f>
-        <v>40000</v>
-      </c>
-      <c r="O17" s="2" t="s">
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>373</v>
-      </c>
-      <c r="B18" s="12">
-        <f>SUM(B13:B17)</f>
-        <v>24268.666666666664</v>
-      </c>
-      <c r="C18" s="12">
-        <f>SUM(C13:C17)</f>
-        <v>24268.666666666664</v>
-      </c>
-      <c r="D18" s="12">
-        <f>SUM(D13:D17)</f>
-        <v>24268.666666666664</v>
-      </c>
-      <c r="E18" s="12">
-        <f>SUM(E13:E17)</f>
-        <v>24268.666666666664</v>
-      </c>
-      <c r="F18" s="12">
-        <f>SUM(F13:F17)</f>
-        <v>24268.666666666664</v>
-      </c>
-      <c r="G18" s="12">
-        <f>SUM(G13:G17)</f>
-        <v>324268.6666666666</v>
-      </c>
-      <c r="H18" s="12">
-        <f>SUM(H13:H17)</f>
-        <v>59059.706666666665</v>
-      </c>
-      <c r="I18" s="12">
-        <f>SUM(I13:I17)</f>
-        <v>59059.706666666665</v>
-      </c>
-      <c r="J18" s="12">
-        <f>SUM(J13:J17)</f>
-        <v>59059.706666666665</v>
-      </c>
-      <c r="K18" s="12">
-        <f>SUM(K13:K17)</f>
-        <v>59059.706666666665</v>
-      </c>
-      <c r="L18" s="12">
-        <f>SUM(L13:L17)</f>
-        <v>30067.173333333332</v>
-      </c>
-      <c r="M18" s="12">
-        <f>SUM(M13:M17)</f>
-        <v>24268.666666666664</v>
-      </c>
-      <c r="N18" s="12">
-        <f>SUM(B18:M18)</f>
-        <v>736186.6666666667</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="B20" s="12">
-        <f>B11-B18</f>
-        <v>5731.333333333336</v>
-      </c>
-      <c r="C20" s="12">
-        <f>C11-C18</f>
-        <v>55731.333333333336</v>
-      </c>
-      <c r="D20" s="12">
-        <f>D11-D18</f>
-        <v>-24268.666666666664</v>
-      </c>
-      <c r="E20" s="12">
-        <f>E11-E18</f>
-        <v>-24268.666666666664</v>
-      </c>
-      <c r="F20" s="12">
-        <f>F11-F18</f>
-        <v>-24268.666666666664</v>
-      </c>
-      <c r="G20" s="12">
-        <f>G11-G18</f>
-        <v>175731.33333333337</v>
-      </c>
-      <c r="H20" s="12">
-        <f>H11-H18</f>
-        <v>-59059.706666666665</v>
-      </c>
-      <c r="I20" s="12">
-        <f>I11-I18</f>
-        <v>-59059.706666666665</v>
-      </c>
-      <c r="J20" s="12">
-        <f>J11-J18</f>
-        <v>-59059.706666666665</v>
-      </c>
-      <c r="K20" s="12">
-        <f>K11-K18</f>
-        <v>-59059.706666666665</v>
-      </c>
-      <c r="L20" s="12">
-        <f>L11-L18</f>
-        <v>-30067.173333333332</v>
-      </c>
-      <c r="M20" s="12">
-        <f>M11-M18</f>
-        <v>-24268.666666666664</v>
-      </c>
-      <c r="N20" s="12">
-        <f>SUM(B20:M20)</f>
-        <v>-126186.6666666666</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="B21" s="8">
+      <c r="B20" s="8">
         <f>'Inputs'!C60</f>
         <v>4041</v>
       </c>
-      <c r="C21" s="8">
-        <f>B22</f>
+      <c r="C20" s="8">
+        <f>B21</f>
         <v>9772.333333333336</v>
       </c>
-      <c r="D21" s="8">
-        <f>C22</f>
+      <c r="D20" s="8">
+        <f>C21</f>
         <v>65503.66666666668</v>
       </c>
-      <c r="E21" s="8">
-        <f>D22</f>
+      <c r="E20" s="8">
+        <f>D21</f>
         <v>41235.000000000015</v>
       </c>
-      <c r="F21" s="8">
-        <f>E22</f>
+      <c r="F20" s="8">
+        <f>E21</f>
         <v>16966.33333333335</v>
       </c>
-      <c r="G21" s="8">
-        <f>F22</f>
+      <c r="G20" s="8">
+        <f>F21</f>
         <v>-7302.333333333314</v>
       </c>
-      <c r="H21" s="8">
-        <f>G22</f>
-        <v>168429.00000000006</v>
-      </c>
-      <c r="I21" s="8">
-        <f>H22</f>
-        <v>109369.2933333334</v>
-      </c>
-      <c r="J21" s="8">
-        <f>I22</f>
-        <v>50309.58666666673</v>
-      </c>
-      <c r="K21" s="8">
-        <f>J22</f>
-        <v>-8750.119999999937</v>
-      </c>
-      <c r="L21" s="8">
-        <f>K22</f>
-        <v>-67809.8266666666</v>
-      </c>
-      <c r="M21" s="8">
-        <f>L22</f>
-        <v>-97876.99999999994</v>
-      </c>
-      <c r="O21" s="2" t="s">
-        <v>378</v>
+      <c r="H20" s="8">
+        <f>G21</f>
+        <v>168179.00000000006</v>
+      </c>
+      <c r="I20" s="8">
+        <f>H21</f>
+        <v>109119.2933333334</v>
+      </c>
+      <c r="J20" s="8">
+        <f>I21</f>
+        <v>50059.58666666673</v>
+      </c>
+      <c r="K20" s="8">
+        <f>J21</f>
+        <v>-9000.119999999937</v>
+      </c>
+      <c r="L20" s="8">
+        <f>K21</f>
+        <v>-68059.8266666666</v>
+      </c>
+      <c r="M20" s="8">
+        <f>L21</f>
+        <v>-98126.99999999994</v>
+      </c>
+      <c r="O20" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="B21" s="12">
+        <f>B20+B19</f>
+        <v>9772.333333333336</v>
+      </c>
+      <c r="C21" s="12">
+        <f>C20+C19</f>
+        <v>65503.66666666668</v>
+      </c>
+      <c r="D21" s="12">
+        <f>D20+D19</f>
+        <v>41235.000000000015</v>
+      </c>
+      <c r="E21" s="12">
+        <f>E20+E19</f>
+        <v>16966.33333333335</v>
+      </c>
+      <c r="F21" s="12">
+        <f>F20+F19</f>
+        <v>-7302.333333333314</v>
+      </c>
+      <c r="G21" s="12">
+        <f>G20+G19</f>
+        <v>168179.00000000006</v>
+      </c>
+      <c r="H21" s="12">
+        <f>H20+H19</f>
+        <v>109119.2933333334</v>
+      </c>
+      <c r="I21" s="12">
+        <f>I20+I19</f>
+        <v>50059.58666666673</v>
+      </c>
+      <c r="J21" s="12">
+        <f>J20+J19</f>
+        <v>-9000.119999999937</v>
+      </c>
+      <c r="K21" s="12">
+        <f>K20+K19</f>
+        <v>-68059.8266666666</v>
+      </c>
+      <c r="L21" s="12">
+        <f>L20+L19</f>
+        <v>-98126.99999999994</v>
+      </c>
+      <c r="M21" s="12">
+        <f>M20+M19</f>
+        <v>-122395.6666666666</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>379</v>
-      </c>
-      <c r="B22" s="12">
-        <f>B21+B20</f>
-        <v>9772.333333333336</v>
-      </c>
-      <c r="C22" s="12">
-        <f>C21+C20</f>
-        <v>65503.66666666668</v>
-      </c>
-      <c r="D22" s="12">
-        <f>D21+D20</f>
-        <v>41235.000000000015</v>
-      </c>
-      <c r="E22" s="12">
-        <f>E21+E20</f>
-        <v>16966.33333333335</v>
-      </c>
-      <c r="F22" s="12">
-        <f>F21+F20</f>
-        <v>-7302.333333333314</v>
-      </c>
-      <c r="G22" s="12">
-        <f>G21+G20</f>
-        <v>168429.00000000006</v>
-      </c>
-      <c r="H22" s="12">
-        <f>H21+H20</f>
-        <v>109369.2933333334</v>
-      </c>
-      <c r="I22" s="12">
-        <f>I21+I20</f>
-        <v>50309.58666666673</v>
-      </c>
-      <c r="J22" s="12">
-        <f>J21+J20</f>
-        <v>-8750.119999999937</v>
-      </c>
-      <c r="K22" s="12">
-        <f>K21+K20</f>
-        <v>-67809.8266666666</v>
-      </c>
-      <c r="L22" s="12">
-        <f>L21+L20</f>
-        <v>-97876.99999999994</v>
-      </c>
-      <c r="M22" s="12">
-        <f>M21+M20</f>
-        <v>-122145.6666666666</v>
+        <v>376</v>
+      </c>
+      <c r="M22" s="14">
+        <f>M21/('Inputs'!C36/'Inputs'!C24)</f>
+        <v>-5.846368181383942</v>
       </c>
       <c r="O22" s="3" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>381</v>
-      </c>
-      <c r="M23" s="14">
-        <f>M22/('Inputs'!C36/'Inputs'!C24)</f>
-        <v>-5.834426647135621</v>
-      </c>
-      <c r="O23" s="3" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
   </sheetData>
@@ -5325,7 +5236,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -5333,13 +5244,13 @@
         <v>240</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>16</v>
@@ -5347,7 +5258,7 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="B3" s="6">
         <v>0</v>
@@ -5359,12 +5270,12 @@
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="B4" s="9">
         <v>1152</v>
@@ -5376,12 +5287,12 @@
         <v>2792</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="B5" s="6">
         <v>400</v>
@@ -5393,12 +5304,12 @@
         <v>900</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="B6" s="8">
         <v>115037.33333333333</v>
@@ -5410,7 +5321,7 @@
         <v>258833.99999999997</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -5427,12 +5338,12 @@
         <v>251224</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="B8" s="9">
         <v>46</v>
@@ -5444,12 +5355,12 @@
         <v>103</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>397</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>398</v>
+        <v>393</v>
       </c>
       <c r="B9" s="5">
         <v>100000</v>
@@ -5461,12 +5372,12 @@
         <v>100000</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>399</v>
+        <v>394</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="B10" s="8">
         <v>136186.6666666667</v>
@@ -5478,12 +5389,12 @@
         <v>-7609.999999999971</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="B11" s="12">
         <v>-36186.666666666686</v>
@@ -5495,29 +5406,29 @@
         <v>107610</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="B13" s="11">
         <v>874</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B14" s="8">
         <v>300000</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -5540,12 +5451,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>279</v>
@@ -5554,105 +5465,105 @@
         <v>15</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>414</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="B9" s="12">
         <v>0</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -5663,7 +5574,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="56" customWidth="1"/>
@@ -5674,1351 +5585,1337 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="C3" s="15">
         <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="C4" s="15">
         <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C5" s="16">
-        <v>136186.66666666674</v>
+        <v>136436.66666666674</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C6" s="15">
-        <v>191224</v>
+        <v>331224</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C7" s="15">
         <v>200000</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C8" s="15">
         <v>50000</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="C9" s="16">
-        <v>55037.33333333333</v>
+        <v>194787.3333333333</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="C10" s="15">
         <v>30000</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="C11" s="15">
         <v>80000</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="C12" s="15">
         <v>110000</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>446</v>
+        <v>441</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="C13" s="15">
         <v>4041</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>448</v>
+        <v>443</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="C14" s="16">
         <v>0.8</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>450</v>
+        <v>445</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="C15" s="15">
         <v>20</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>451</v>
+        <v>446</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="C16" s="15">
         <v>1</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>452</v>
+        <v>447</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="C17" s="15">
         <v>6</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="C18" s="15">
         <v>16</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>454</v>
+        <v>449</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>449</v>
+        <v>444</v>
       </c>
       <c r="C19" s="15">
         <v>96</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>455</v>
+        <v>450</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="C20" s="15">
         <v>50000</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C21" s="15">
-        <v>600000</v>
+        <v>599750</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C22" s="15">
         <v>300000</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>460</v>
+        <v>455</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C23" s="15">
         <v>100000</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C24" s="15">
-        <v>60000</v>
+        <v>99750</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C25" s="15">
-        <v>40000</v>
+        <v>100000</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C26" s="15">
-        <v>100000</v>
+        <v>453</v>
+      </c>
+      <c r="C26" s="16">
+        <v>104962.66666666667</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C27" s="16">
-        <v>104962.66666666667</v>
+        <v>453</v>
+      </c>
+      <c r="C27" s="15">
+        <v>266</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C28" s="15">
-        <v>80</v>
+        <v>399</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C29" s="15">
-        <v>213</v>
+        <v>134</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C30" s="15">
-        <v>320</v>
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C31" s="15">
-        <v>187</v>
+        <v>400</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>469</v>
+        <v>464</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C32" s="15">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>470</v>
+        <v>465</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C33" s="15">
-        <v>100</v>
+        <v>453</v>
+      </c>
+      <c r="C33" s="16">
+        <v>262.4066666666667</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>471</v>
+        <v>466</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C34" s="16">
-        <v>262.4066666666667</v>
+        <v>453</v>
+      </c>
+      <c r="C34" s="15">
+        <v>750</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>472</v>
+        <v>467</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C35" s="15">
-        <v>750</v>
+        <v>453</v>
+      </c>
+      <c r="C35" s="16">
+        <v>93.5</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>473</v>
+        <v>468</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C36" s="16">
-        <v>93.5</v>
+        <v>287.5933333333333</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C37" s="16">
-        <v>287.5933333333333</v>
+        <v>453</v>
+      </c>
+      <c r="C37" s="15">
+        <v>40000</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C38" s="15">
-        <v>40000</v>
+        <v>4</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C39" s="15">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C40" s="15">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C41" s="15">
-        <v>400</v>
+        <v>40000</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C42" s="15">
-        <v>40000</v>
+        <v>453</v>
+      </c>
+      <c r="C42" s="16">
+        <v>5.24</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C43" s="16">
-        <v>5.24</v>
+        <v>453</v>
+      </c>
+      <c r="C43" s="15">
+        <v>6</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C44" s="15">
-        <v>6</v>
+        <v>453</v>
+      </c>
+      <c r="C44" s="16">
+        <v>66.66666666666667</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C45" s="16">
-        <v>66.66666666666667</v>
+        <v>736186.6666666667</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C46" s="16">
-        <v>736186.6666666667</v>
+        <v>115037.33333333333</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C47" s="16">
-        <v>115037.33333333333</v>
+        <v>453</v>
+      </c>
+      <c r="C47" s="15">
+        <v>331224</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C48" s="15">
-        <v>331224</v>
+        <v>453</v>
+      </c>
+      <c r="C48" s="16">
+        <v>136186.6666666667</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>458</v>
-      </c>
-      <c r="C49" s="16">
-        <v>136186.6666666667</v>
+        <v>453</v>
+      </c>
+      <c r="C49" s="15">
+        <v>300000</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C50" s="15">
-        <v>300000</v>
+        <v>2</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C51" s="15">
-        <v>2</v>
+        <v>150000</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C52" s="15">
-        <v>150000</v>
+        <v>142467</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C53" s="15">
-        <v>142467</v>
+        <v>95767</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C54" s="15">
-        <v>95767</v>
+        <v>55</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C55" s="15">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C56" s="15">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C57" s="15">
-        <v>15</v>
+        <v>251224</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C58" s="15">
-        <v>251224</v>
+        <v>151200</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C59" s="15">
-        <v>151200</v>
+        <v>51000</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C60" s="15">
-        <v>51000</v>
+        <v>3674</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C61" s="15">
-        <v>3674</v>
+        <v>27000</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C62" s="15">
-        <v>27000</v>
+        <v>10000</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C63" s="15">
-        <v>10000</v>
+        <v>8350</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C64" s="15">
-        <v>8350</v>
+        <v>0</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="C65" s="15">
         <v>0</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>458</v>
+        <v>499</v>
       </c>
       <c r="C66" s="15">
-        <v>0</v>
+        <v>874</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C67" s="15">
-        <v>874</v>
+        <v>10000</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C68" s="15">
-        <v>10000</v>
+        <v>300000</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C69" s="15">
-        <v>300000</v>
+        <v>46</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C70" s="15">
-        <v>46</v>
+        <v>100</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C71" s="15">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C72" s="15">
-        <v>103</v>
+        <v>1152</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C73" s="15">
-        <v>1152</v>
+        <v>400</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C74" s="15">
-        <v>400</v>
+        <v>1152</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C75" s="15">
-        <v>1152</v>
+        <v>100000</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C76" s="15">
-        <v>100000</v>
+        <v>0</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C77" s="15">
-        <v>0</v>
+        <v>251224</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C78" s="15">
-        <v>251224</v>
+        <v>874</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C79" s="15">
-        <v>874</v>
+        <v>1552</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C80" s="15">
-        <v>1552</v>
+        <v>100000</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C81" s="15">
-        <v>100000</v>
+        <v>2</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C82" s="15">
-        <v>2</v>
+        <v>251224</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C83" s="15">
-        <v>251224</v>
+        <v>900</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C84" s="15">
-        <v>900</v>
+        <v>2792</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>523</v>
+        <v>518</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C85" s="15">
-        <v>2792</v>
+        <v>100000</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C86" s="15">
-        <v>100000</v>
+        <v>3</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>525</v>
+        <v>520</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C87" s="15">
-        <v>3</v>
+        <v>251224</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>526</v>
+        <v>521</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="C88" s="15">
-        <v>251224</v>
+        <v>499</v>
+      </c>
+      <c r="C88" s="16">
+        <v>-36186.666666666686</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>527</v>
+        <v>522</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C89" s="16">
-        <v>-36186.666666666686</v>
+        <v>100132.5733333333</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>528</v>
+        <v>523</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="C90" s="16">
-        <v>100132.5733333333</v>
+        <v>499</v>
+      </c>
+      <c r="C90" s="15">
+        <v>107610</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>529</v>
+        <v>524</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="C91" s="15">
-        <v>107610</v>
+        <v>499</v>
+      </c>
+      <c r="C91" s="16">
+        <v>115037.33333333333</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
-        <v>530</v>
+        <v>525</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C92" s="16">
-        <v>115037.33333333333</v>
+        <v>251356.5733333333</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>531</v>
+        <v>526</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C93" s="16">
-        <v>251356.5733333333</v>
+        <v>258833.99999999997</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
-        <v>532</v>
+        <v>527</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C94" s="16">
-        <v>258833.99999999997</v>
+        <v>136186.6666666667</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C95" s="16">
-        <v>136186.6666666667</v>
+        <v>-132.57333333330462</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
-        <v>534</v>
+        <v>529</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>505</v>
+        <v>499</v>
       </c>
       <c r="C96" s="16">
-        <v>-132.57333333330462</v>
+        <v>-7609.999999999971</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
-        <v>535</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>505</v>
-      </c>
-      <c r="C97" s="16">
-        <v>-7609.999999999971</v>
-      </c>
-      <c r="D97" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The SEFA loan of $150,000 sits inside the ask
Ben, 15 September 2026 (evening): no grant carries the running cost; a loan
does. LOAN_ASK_AUD enters the asks as a loan, grants and loans are summed
apart, and the funder workbook and sheet canon read the same ask.
</commit_message>
<xml_diff>
--- a/deliverables/finance/funder-model/goods-funder-model-2026-09-15.xlsx
+++ b/deliverables/finance/funder-model/goods-funder-model-2026-09-15.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="531">
   <si>
     <t>Goods on Country, financial model for funders</t>
   </si>
@@ -842,7 +842,7 @@
     <t>Organisation: running it, and the freight and facilitation it absorbs</t>
   </si>
   <si>
-    <t>Nobody is asked for this line (Ben, 15 September 2026). It is carried by 400 beds at the contribution, and by trade beyond them.</t>
+    <t>No grant is asked for this line. The $150,000 SEFA loan inside the ask carries the first-year gap (Ben, 15 September 2026); the rest is carried by 400 beds at the contribution.</t>
   </si>
   <si>
     <t>The year needs</t>
@@ -914,6 +914,18 @@
     <t>Ben wrote $100,000 on 10 September and ruled it counts as beds, 133 at $750. The ask has not been sent.</t>
   </si>
   <si>
+    <t>SEFA, Backing the Bold</t>
+  </si>
+  <si>
+    <t>operating</t>
+  </si>
+  <si>
+    <t>not counted</t>
+  </si>
+  <si>
+    <t>Ben, 15 September 2026: the first-year running gap is carried by a SEFA loan of $150,000, inside the ask, repaid from the $288 each bed hands back. Jay's steer for QBE 2026 is philanthropy that unlocks capital, and this is the capital. EOI drafted; Joel Bird reviews the financials before it goes.</t>
+  </si>
+  <si>
     <t>Dusseldorp Forum</t>
   </si>
   <si>
@@ -923,18 +935,6 @@
     <t>Top-up. $50,000 is our number, nothing from the funder yet.</t>
   </si>
   <si>
-    <t>SEFA, Backing the Bold, up to</t>
-  </si>
-  <si>
-    <t>not applied</t>
-  </si>
-  <si>
-    <t>not counted</t>
-  </si>
-  <si>
-    <t>A loan. It is never counted in the ask, the gap or the beds covered. Debt needs a repayment source and an entity, both open.</t>
-  </si>
-  <si>
     <t>Totals</t>
   </si>
   <si>
@@ -944,7 +944,7 @@
     <t>No Snow, no Dusseldorp</t>
   </si>
   <si>
-    <t>Four lines, all grants. Dusseldorp and SEFA are outside the ask.</t>
+    <t>Four grants and one loan. Dusseldorp is outside the ask.</t>
   </si>
   <si>
     <t>Secured</t>
@@ -1004,7 +1004,7 @@
     <t>Beds at the contribution, after making, freight and facilitation.</t>
   </si>
   <si>
-    <t>Against running alone, because the contribution already carries the freight and facilitation. No grant goes against this line; it is the running short that trade or debt has to cover.</t>
+    <t>Against running alone, because the contribution already carries the freight and facilitation. No grant goes against this line; the SEFA loan inside the ask carries it.</t>
   </si>
   <si>
     <t>Monthly cash, July 2026 to June 2027. A scenario laid out from the Inputs sheet. Nobody has forecast these months. Built 2026-09-15.</t>
@@ -1076,10 +1076,10 @@
     <t>Scenario month only. No receipt date exists. Invited; SmartyGrants closes 9 October, board late November. Ben, 15 September 2026: buys beds, not the running cost.</t>
   </si>
   <si>
-    <t>Loan drawn (SEFA)</t>
-  </si>
-  <si>
-    <t>Zero until applied for. Up to the Inputs loan cap; no rate or term is set.</t>
+    <t>Loan drawn (SEFA, inside the ask)</t>
+  </si>
+  <si>
+    <t>Scenario month only. Ben, 15 September 2026: $150,000 inside the ask, repaid from the contribution. EOI drafted, unsent; Joel Bird reviews first.</t>
   </si>
   <si>
     <t>Bed sales to buyers</t>
@@ -1392,6 +1392,9 @@
   </si>
   <si>
     <t>ASKS[3].amountAud</t>
+  </si>
+  <si>
+    <t>ASKS[4].amountAud</t>
   </si>
   <si>
     <t>BEDS_AT_COST_AUD</t>
@@ -3816,11 +3819,12 @@
         <v>331224</v>
       </c>
       <c r="C6" s="8">
-        <v>0</v>
+        <f>SUM(B15)</f>
+        <v>150000</v>
       </c>
       <c r="D6" s="8">
         <f>MAX(0,B6-C6)</f>
-        <v>331224</v>
+        <v>181224</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>274</v>
@@ -3836,11 +3840,11 @@
       </c>
       <c r="C7" s="12">
         <f>SUM(C4,C5,C6)</f>
-        <v>599750</v>
+        <v>749750</v>
       </c>
       <c r="D7" s="12">
         <f>B7-C7</f>
-        <v>136436.66666666674</v>
+        <v>-13563.333333333256</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>276</v>
@@ -3979,44 +3983,44 @@
       <c r="A15" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="B15" s="5">
-        <v>50000</v>
+      <c r="B15" s="13">
+        <v>150000</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>89</v>
+        <v>299</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="E15" s="6">
-        <f>FLOOR(B15/'Inputs'!C4,1)</f>
-        <v>66</v>
+      <c r="E15" s="2" t="s">
+        <v>300</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>301</v>
-      </c>
-      <c r="B16" s="13">
-        <v>200000</v>
+        <v>302</v>
+      </c>
+      <c r="B16" s="5">
+        <v>50000</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="E16" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="E16" s="6">
+        <f>FLOOR(B16/'Inputs'!C4,1)</f>
+        <v>66</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>299</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>304</v>
@@ -4061,8 +4065,8 @@
         <v>266</v>
       </c>
       <c r="B20" s="12">
-        <f>SUM(B11,B12,B13,B14)</f>
-        <v>599750</v>
+        <f>SUM(B11,B12,B13,B14,B15)</f>
+        <v>749750</v>
       </c>
       <c r="C20" s="12">
         <f>SUM(B11,B12,B13)</f>
@@ -4092,7 +4096,7 @@
       </c>
       <c r="B22" s="12">
         <f>B7-B20</f>
-        <v>136436.66666666674</v>
+        <v>-13563.333333333256</v>
       </c>
       <c r="C22" s="12">
         <f>B7-C20</f>
@@ -4155,7 +4159,7 @@
         <v>319</v>
       </c>
       <c r="B26" s="8">
-        <v>331224</v>
+        <v>181224</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>320</v>
@@ -4542,7 +4546,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="5">
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="H8" s="5">
         <v>0</v>
@@ -4564,7 +4568,7 @@
       </c>
       <c r="N8" s="5">
         <f>SUM(B8:M8)</f>
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="O8" s="2" t="s">
         <v>353</v>
@@ -4646,7 +4650,7 @@
       </c>
       <c r="G10" s="12">
         <f>SUM(G4:G9)</f>
-        <v>499750</v>
+        <v>649750</v>
       </c>
       <c r="H10" s="12">
         <f>SUM(H4:H9)</f>
@@ -5060,7 +5064,7 @@
       </c>
       <c r="G19" s="12">
         <f>G10-G17</f>
-        <v>175481.33333333337</v>
+        <v>325481.3333333334</v>
       </c>
       <c r="H19" s="12">
         <f>H10-H17</f>
@@ -5088,7 +5092,7 @@
       </c>
       <c r="N19" s="12">
         <f>SUM(B19:M19)</f>
-        <v>-126436.6666666666</v>
+        <v>23563.3333333334</v>
       </c>
       <c r="O19" s="3" t="s">
         <v>371</v>
@@ -5124,27 +5128,27 @@
       </c>
       <c r="H20" s="8">
         <f>G21</f>
-        <v>168179.00000000006</v>
+        <v>318179.0000000001</v>
       </c>
       <c r="I20" s="8">
         <f>H21</f>
-        <v>109119.2933333334</v>
+        <v>259119.29333333345</v>
       </c>
       <c r="J20" s="8">
         <f>I21</f>
-        <v>50059.58666666673</v>
+        <v>200059.5866666668</v>
       </c>
       <c r="K20" s="8">
         <f>J21</f>
-        <v>-9000.119999999937</v>
+        <v>140999.88000000012</v>
       </c>
       <c r="L20" s="8">
         <f>K21</f>
-        <v>-68059.8266666666</v>
+        <v>81940.17333333346</v>
       </c>
       <c r="M20" s="8">
         <f>L21</f>
-        <v>-98126.99999999994</v>
+        <v>51873.000000000124</v>
       </c>
       <c r="O20" s="2" t="s">
         <v>373</v>
@@ -5176,31 +5180,31 @@
       </c>
       <c r="G21" s="12">
         <f>G20+G19</f>
-        <v>168179.00000000006</v>
+        <v>318179.0000000001</v>
       </c>
       <c r="H21" s="12">
         <f>H20+H19</f>
-        <v>109119.2933333334</v>
+        <v>259119.29333333345</v>
       </c>
       <c r="I21" s="12">
         <f>I20+I19</f>
-        <v>50059.58666666673</v>
+        <v>200059.5866666668</v>
       </c>
       <c r="J21" s="12">
         <f>J20+J19</f>
-        <v>-9000.119999999937</v>
+        <v>140999.88000000012</v>
       </c>
       <c r="K21" s="12">
         <f>K20+K19</f>
-        <v>-68059.8266666666</v>
+        <v>81940.17333333346</v>
       </c>
       <c r="L21" s="12">
         <f>L20+L19</f>
-        <v>-98126.99999999994</v>
+        <v>51873.000000000124</v>
       </c>
       <c r="M21" s="12">
         <f>M20+M19</f>
-        <v>-122395.6666666666</v>
+        <v>27604.33333333346</v>
       </c>
       <c r="O21" s="3" t="s">
         <v>375</v>
@@ -5212,7 +5216,7 @@
       </c>
       <c r="M22" s="14">
         <f>M21/('Inputs'!C36/'Inputs'!C24)</f>
-        <v>-5.846368181383942</v>
+        <v>1.3185523676081965</v>
       </c>
       <c r="O22" s="3" t="s">
         <v>377</v>
@@ -5574,7 +5578,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="56" customWidth="1"/>
@@ -5638,7 +5642,7 @@
         <v>432</v>
       </c>
       <c r="C5" s="16">
-        <v>136436.66666666674</v>
+        <v>-13563.333333333256</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>429</v>
@@ -5652,7 +5656,7 @@
         <v>432</v>
       </c>
       <c r="C6" s="15">
-        <v>331224</v>
+        <v>181224</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>429</v>
@@ -5862,7 +5866,7 @@
         <v>453</v>
       </c>
       <c r="C21" s="15">
-        <v>599750</v>
+        <v>749750</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>429</v>
@@ -5931,8 +5935,8 @@
       <c r="B26" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C26" s="16">
-        <v>104962.66666666667</v>
+      <c r="C26" s="15">
+        <v>150000</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>429</v>
@@ -5945,8 +5949,8 @@
       <c r="B27" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C27" s="15">
-        <v>266</v>
+      <c r="C27" s="16">
+        <v>104962.66666666667</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>429</v>
@@ -5960,7 +5964,7 @@
         <v>453</v>
       </c>
       <c r="C28" s="15">
-        <v>399</v>
+        <v>266</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>429</v>
@@ -5974,7 +5978,7 @@
         <v>453</v>
       </c>
       <c r="C29" s="15">
-        <v>134</v>
+        <v>399</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>429</v>
@@ -5988,7 +5992,7 @@
         <v>453</v>
       </c>
       <c r="C30" s="15">
-        <v>1</v>
+        <v>134</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>429</v>
@@ -6002,7 +6006,7 @@
         <v>453</v>
       </c>
       <c r="C31" s="15">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>429</v>
@@ -6016,7 +6020,7 @@
         <v>453</v>
       </c>
       <c r="C32" s="15">
-        <v>100</v>
+        <v>400</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>429</v>
@@ -6029,8 +6033,8 @@
       <c r="B33" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C33" s="16">
-        <v>262.4066666666667</v>
+      <c r="C33" s="15">
+        <v>100</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>429</v>
@@ -6043,8 +6047,8 @@
       <c r="B34" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C34" s="15">
-        <v>750</v>
+      <c r="C34" s="16">
+        <v>262.4066666666667</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>429</v>
@@ -6057,8 +6061,8 @@
       <c r="B35" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C35" s="16">
-        <v>93.5</v>
+      <c r="C35" s="15">
+        <v>750</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>429</v>
@@ -6072,7 +6076,7 @@
         <v>453</v>
       </c>
       <c r="C36" s="16">
-        <v>287.5933333333333</v>
+        <v>93.5</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>429</v>
@@ -6085,8 +6089,8 @@
       <c r="B37" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C37" s="15">
-        <v>40000</v>
+      <c r="C37" s="16">
+        <v>287.5933333333333</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>429</v>
@@ -6100,7 +6104,7 @@
         <v>453</v>
       </c>
       <c r="C38" s="15">
-        <v>4</v>
+        <v>40000</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>429</v>
@@ -6114,7 +6118,7 @@
         <v>453</v>
       </c>
       <c r="C39" s="15">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>429</v>
@@ -6128,7 +6132,7 @@
         <v>453</v>
       </c>
       <c r="C40" s="15">
-        <v>400</v>
+        <v>100</v>
       </c>
       <c r="D40" s="2" t="s">
         <v>429</v>
@@ -6142,7 +6146,7 @@
         <v>453</v>
       </c>
       <c r="C41" s="15">
-        <v>40000</v>
+        <v>400</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>429</v>
@@ -6155,8 +6159,8 @@
       <c r="B42" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C42" s="16">
-        <v>5.24</v>
+      <c r="C42" s="15">
+        <v>40000</v>
       </c>
       <c r="D42" s="2" t="s">
         <v>429</v>
@@ -6169,8 +6173,8 @@
       <c r="B43" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C43" s="15">
-        <v>6</v>
+      <c r="C43" s="16">
+        <v>5.24</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>429</v>
@@ -6183,8 +6187,8 @@
       <c r="B44" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C44" s="16">
-        <v>66.66666666666667</v>
+      <c r="C44" s="15">
+        <v>6</v>
       </c>
       <c r="D44" s="2" t="s">
         <v>429</v>
@@ -6198,7 +6202,7 @@
         <v>453</v>
       </c>
       <c r="C45" s="16">
-        <v>736186.6666666667</v>
+        <v>66.66666666666667</v>
       </c>
       <c r="D45" s="2" t="s">
         <v>429</v>
@@ -6212,7 +6216,7 @@
         <v>453</v>
       </c>
       <c r="C46" s="16">
-        <v>115037.33333333333</v>
+        <v>736186.6666666667</v>
       </c>
       <c r="D46" s="2" t="s">
         <v>429</v>
@@ -6225,8 +6229,8 @@
       <c r="B47" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C47" s="15">
-        <v>331224</v>
+      <c r="C47" s="16">
+        <v>115037.33333333333</v>
       </c>
       <c r="D47" s="2" t="s">
         <v>429</v>
@@ -6239,8 +6243,8 @@
       <c r="B48" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C48" s="16">
-        <v>136186.6666666667</v>
+      <c r="C48" s="15">
+        <v>331224</v>
       </c>
       <c r="D48" s="2" t="s">
         <v>429</v>
@@ -6253,8 +6257,8 @@
       <c r="B49" s="2" t="s">
         <v>453</v>
       </c>
-      <c r="C49" s="15">
-        <v>300000</v>
+      <c r="C49" s="16">
+        <v>136186.6666666667</v>
       </c>
       <c r="D49" s="2" t="s">
         <v>429</v>
@@ -6268,7 +6272,7 @@
         <v>453</v>
       </c>
       <c r="C50" s="15">
-        <v>2</v>
+        <v>300000</v>
       </c>
       <c r="D50" s="2" t="s">
         <v>429</v>
@@ -6282,7 +6286,7 @@
         <v>453</v>
       </c>
       <c r="C51" s="15">
-        <v>150000</v>
+        <v>2</v>
       </c>
       <c r="D51" s="2" t="s">
         <v>429</v>
@@ -6296,7 +6300,7 @@
         <v>453</v>
       </c>
       <c r="C52" s="15">
-        <v>142467</v>
+        <v>150000</v>
       </c>
       <c r="D52" s="2" t="s">
         <v>429</v>
@@ -6310,7 +6314,7 @@
         <v>453</v>
       </c>
       <c r="C53" s="15">
-        <v>95767</v>
+        <v>142467</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>429</v>
@@ -6324,7 +6328,7 @@
         <v>453</v>
       </c>
       <c r="C54" s="15">
-        <v>55</v>
+        <v>95767</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>429</v>
@@ -6338,7 +6342,7 @@
         <v>453</v>
       </c>
       <c r="C55" s="15">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="D55" s="2" t="s">
         <v>429</v>
@@ -6352,7 +6356,7 @@
         <v>453</v>
       </c>
       <c r="C56" s="15">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="D56" s="2" t="s">
         <v>429</v>
@@ -6366,7 +6370,7 @@
         <v>453</v>
       </c>
       <c r="C57" s="15">
-        <v>251224</v>
+        <v>15</v>
       </c>
       <c r="D57" s="2" t="s">
         <v>429</v>
@@ -6380,7 +6384,7 @@
         <v>453</v>
       </c>
       <c r="C58" s="15">
-        <v>151200</v>
+        <v>251224</v>
       </c>
       <c r="D58" s="2" t="s">
         <v>429</v>
@@ -6394,7 +6398,7 @@
         <v>453</v>
       </c>
       <c r="C59" s="15">
-        <v>51000</v>
+        <v>151200</v>
       </c>
       <c r="D59" s="2" t="s">
         <v>429</v>
@@ -6408,7 +6412,7 @@
         <v>453</v>
       </c>
       <c r="C60" s="15">
-        <v>3674</v>
+        <v>51000</v>
       </c>
       <c r="D60" s="2" t="s">
         <v>429</v>
@@ -6422,7 +6426,7 @@
         <v>453</v>
       </c>
       <c r="C61" s="15">
-        <v>27000</v>
+        <v>3674</v>
       </c>
       <c r="D61" s="2" t="s">
         <v>429</v>
@@ -6436,7 +6440,7 @@
         <v>453</v>
       </c>
       <c r="C62" s="15">
-        <v>10000</v>
+        <v>27000</v>
       </c>
       <c r="D62" s="2" t="s">
         <v>429</v>
@@ -6450,7 +6454,7 @@
         <v>453</v>
       </c>
       <c r="C63" s="15">
-        <v>8350</v>
+        <v>10000</v>
       </c>
       <c r="D63" s="2" t="s">
         <v>429</v>
@@ -6464,7 +6468,7 @@
         <v>453</v>
       </c>
       <c r="C64" s="15">
-        <v>0</v>
+        <v>8350</v>
       </c>
       <c r="D64" s="2" t="s">
         <v>429</v>
@@ -6489,10 +6493,10 @@
         <v>498</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>499</v>
+        <v>453</v>
       </c>
       <c r="C66" s="15">
-        <v>874</v>
+        <v>0</v>
       </c>
       <c r="D66" s="2" t="s">
         <v>429</v>
@@ -6500,13 +6504,13 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>499</v>
-      </c>
       <c r="C67" s="15">
-        <v>10000</v>
+        <v>874</v>
       </c>
       <c r="D67" s="2" t="s">
         <v>429</v>
@@ -6517,10 +6521,10 @@
         <v>501</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C68" s="15">
-        <v>300000</v>
+        <v>10000</v>
       </c>
       <c r="D68" s="2" t="s">
         <v>429</v>
@@ -6531,10 +6535,10 @@
         <v>502</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C69" s="15">
-        <v>46</v>
+        <v>300000</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>429</v>
@@ -6545,10 +6549,10 @@
         <v>503</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C70" s="15">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="D70" s="2" t="s">
         <v>429</v>
@@ -6559,10 +6563,10 @@
         <v>504</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C71" s="15">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D71" s="2" t="s">
         <v>429</v>
@@ -6573,10 +6577,10 @@
         <v>505</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C72" s="15">
-        <v>1152</v>
+        <v>103</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>429</v>
@@ -6587,10 +6591,10 @@
         <v>506</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C73" s="15">
-        <v>400</v>
+        <v>1152</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>429</v>
@@ -6601,10 +6605,10 @@
         <v>507</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C74" s="15">
-        <v>1152</v>
+        <v>400</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>429</v>
@@ -6615,10 +6619,10 @@
         <v>508</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C75" s="15">
-        <v>100000</v>
+        <v>1152</v>
       </c>
       <c r="D75" s="2" t="s">
         <v>429</v>
@@ -6629,10 +6633,10 @@
         <v>509</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C76" s="15">
-        <v>0</v>
+        <v>100000</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>429</v>
@@ -6643,10 +6647,10 @@
         <v>510</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C77" s="15">
-        <v>251224</v>
+        <v>0</v>
       </c>
       <c r="D77" s="2" t="s">
         <v>429</v>
@@ -6657,10 +6661,10 @@
         <v>511</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C78" s="15">
-        <v>874</v>
+        <v>251224</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>429</v>
@@ -6671,10 +6675,10 @@
         <v>512</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C79" s="15">
-        <v>1552</v>
+        <v>874</v>
       </c>
       <c r="D79" s="2" t="s">
         <v>429</v>
@@ -6685,10 +6689,10 @@
         <v>513</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C80" s="15">
-        <v>100000</v>
+        <v>1552</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>429</v>
@@ -6699,10 +6703,10 @@
         <v>514</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C81" s="15">
-        <v>2</v>
+        <v>100000</v>
       </c>
       <c r="D81" s="2" t="s">
         <v>429</v>
@@ -6713,10 +6717,10 @@
         <v>515</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C82" s="15">
-        <v>251224</v>
+        <v>2</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>429</v>
@@ -6727,10 +6731,10 @@
         <v>516</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C83" s="15">
-        <v>900</v>
+        <v>251224</v>
       </c>
       <c r="D83" s="2" t="s">
         <v>429</v>
@@ -6741,10 +6745,10 @@
         <v>517</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C84" s="15">
-        <v>2792</v>
+        <v>900</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>429</v>
@@ -6755,10 +6759,10 @@
         <v>518</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C85" s="15">
-        <v>100000</v>
+        <v>2792</v>
       </c>
       <c r="D85" s="2" t="s">
         <v>429</v>
@@ -6769,10 +6773,10 @@
         <v>519</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C86" s="15">
-        <v>3</v>
+        <v>100000</v>
       </c>
       <c r="D86" s="2" t="s">
         <v>429</v>
@@ -6783,10 +6787,10 @@
         <v>520</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C87" s="15">
-        <v>251224</v>
+        <v>3</v>
       </c>
       <c r="D87" s="2" t="s">
         <v>429</v>
@@ -6797,10 +6801,10 @@
         <v>521</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="C88" s="16">
-        <v>-36186.666666666686</v>
+        <v>500</v>
+      </c>
+      <c r="C88" s="15">
+        <v>251224</v>
       </c>
       <c r="D88" s="2" t="s">
         <v>429</v>
@@ -6811,10 +6815,10 @@
         <v>522</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C89" s="16">
-        <v>100132.5733333333</v>
+        <v>-36186.666666666686</v>
       </c>
       <c r="D89" s="2" t="s">
         <v>429</v>
@@ -6825,10 +6829,10 @@
         <v>523</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="C90" s="15">
-        <v>107610</v>
+        <v>500</v>
+      </c>
+      <c r="C90" s="16">
+        <v>100132.5733333333</v>
       </c>
       <c r="D90" s="2" t="s">
         <v>429</v>
@@ -6839,10 +6843,10 @@
         <v>524</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>499</v>
-      </c>
-      <c r="C91" s="16">
-        <v>115037.33333333333</v>
+        <v>500</v>
+      </c>
+      <c r="C91" s="15">
+        <v>107610</v>
       </c>
       <c r="D91" s="2" t="s">
         <v>429</v>
@@ -6853,10 +6857,10 @@
         <v>525</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C92" s="16">
-        <v>251356.5733333333</v>
+        <v>115037.33333333333</v>
       </c>
       <c r="D92" s="2" t="s">
         <v>429</v>
@@ -6867,10 +6871,10 @@
         <v>526</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C93" s="16">
-        <v>258833.99999999997</v>
+        <v>251356.5733333333</v>
       </c>
       <c r="D93" s="2" t="s">
         <v>429</v>
@@ -6881,10 +6885,10 @@
         <v>527</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C94" s="16">
-        <v>136186.6666666667</v>
+        <v>258833.99999999997</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>429</v>
@@ -6895,10 +6899,10 @@
         <v>528</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C95" s="16">
-        <v>-132.57333333330462</v>
+        <v>136186.6666666667</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>429</v>
@@ -6909,12 +6913,26 @@
         <v>529</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C96" s="16">
+        <v>-132.57333333330462</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C97" s="16">
         <v>-7609.999999999971</v>
       </c>
-      <c r="D96" s="2" t="s">
+      <c r="D97" s="2" t="s">
         <v>429</v>
       </c>
     </row>

</xml_diff>